<commit_message>
Recapture screenshots and sample run with vaulted demo evidence
Screenshots now show verified vault badges, the populated Evidence pane
and the corrected rejection text. The sample-run README no longer says
the vault column is always 'No', and describes oscal.json as
OSCAL-inspired and unvalidated, matching the main README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEsj6q59UZDr5R4xFobVsY
</commit_message>
<xml_diff>
--- a/docs/sample-run/racm.xlsx
+++ b/docs/sample-run/racm.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8b43885d-7a9f-400e-ae04-363d14a09d22</t>
+          <t>67d3b1ae-7dd2-49fb-b15f-3fce45051998</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-26T00:41:02+00:00</t>
+          <t>2026-09-26T01:00:45+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: phase table and sample run for the audit model
Regenerated the sample-run exports from a DEMO_MODE API run (three
gates approved) and described the new columns and report section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEsj6q59UZDr5R4xFobVsY
</commit_message>
<xml_diff>
--- a/docs/sample-run/racm.xlsx
+++ b/docs/sample-run/racm.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,32 +434,107 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Likelihood</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rating Rationale</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Regulatory Mapping</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Control ID</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Control Description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Control Owner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Key Control</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Assertions / Objectives</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>IPE</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ToD Steps</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ToE Steps</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Substantive Steps</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Population Source</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Population Completeness</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Sample Size</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling Method</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Period of Reliance</t>
         </is>
       </c>
     </row>
@@ -471,37 +546,100 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[DEMO DATA] Unauthorized access to IAM or S3 resources.</t>
+          <t>[DEMO DATA] Unauthorised access to AWS resources through weak or unreviewed IAM credentials.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CIS AWS Foundations (demo mapping)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Console credentials are reachable from the internet; misuse would expose customer data and infrastructure.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NIST SP 800-53 IA-5 (demo mapping), NIST SP 800-53 AC-2 (demo mapping), ISO/IEC 27001:2022 A.5.17 (demo mapping)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>CTRL-01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Enforce a strict IAM password policy.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Verify that a password policy is defined in IAM. (Expect: Password policy exists and is configured.)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Run the get_iam_password_policy tool. (Expect: Minimum length and complexity match the organisation's standard.)</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Compare the policy values with the benchmark. (Expect: Each value meets or exceeds the benchmark.)</t>
+          <t>The IAM account password policy enforces the organisation's minimum length and complexity.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cloud Platform Engineering Lead</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Preventive</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Access to programs and data; Confidentiality</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Run the get_iam_password_policy tool and compare each setting with the organisation's standard. (Expect: Minimum length of at least 14 and the complexity rules are configured (design and implementation).)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Test of one: the configuration read, plus reliance on change-management ITGCs over IAM configuration or AWS Config history covering the period. (Expect: No change weakened the policy during the period of reliance.)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>If the policy was weaker at any time, list console users whose password was last set before the policy took effect. (Expect: Affected users are identified for follow-up.)</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Test of one</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>[DEMO DATA] 2026-01-01 to 2026-12-31 (assumed)</t>
         </is>
       </c>
     </row>
@@ -513,35 +651,223 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[DEMO DATA] Unauthorized access to IAM or S3 resources.</t>
+          <t>[DEMO DATA] Unauthorised access to AWS resources through weak or unreviewed IAM credentials.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CIS AWS Foundations (demo mapping)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Console credentials are reachable from the internet; misuse would expose customer data and infrastructure.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NIST SP 800-53 IA-5 (demo mapping), NIST SP 800-53 AC-2 (demo mapping), ISO/IEC 27001:2022 A.5.17 (demo mapping)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CTRL-03</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Quarterly review of IAM users with console access: the reviewer signs off and inappropriate access is removed.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Security Operations Manager</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>IT-dependent manual</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Detective</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Access to programs and data</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>IAM credential report used as the review listing</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Walk through one review: listing source, reviewer, sign-off and removal of access. (Expect: The review covers all console users and removals are tracked to completion.)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>For each sampled quarter, inspect the signed review and the tickets for access removed. (Expect: Each review is signed off on time and every flagged user was removed.)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Compare leavers reported by HR for the period with active IAM users. (Expect: No leaver retains console access.)</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Quarterly access reviews performed in the period</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Agree the IAM credential report used by each review to a report re-run by the auditor for the same date (IPE completeness and accuracy).</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Random</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>[DEMO DATA] 2026-01-01 to 2026-12-31 (assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RISK-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[DEMO DATA] Customer data in S3 is exposed publicly.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A single public ACL exposes a bucket to the internet, and the buckets hold customer data.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CIS AWS Foundations Benchmark, S3 section (demo mapping), NIST SP 800-53 AC-3 (demo mapping)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>CTRL-02</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Block public access on S3 buckets.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Confirm account-level S3 Block Public Access is configured. (Expect: All four Block Public Access settings are on.)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>List buckets and inspect each bucket's public access block. (Expect: No bucket allows public ACLs or policies.)</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>S3 Block Public Access is enabled at account level and on every bucket.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cloud Platform Engineering Lead</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Preventive</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Confidentiality</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Run the list_public_s3_buckets tool and inspect account- and bucket-level Block Public Access. (Expect: All four Block Public Access settings are on for the account and each bucket.)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Inspect AWS Config history for Block Public Access changes on each bucket during the period. (Expect: No bucket allowed public ACLs or policies at any time in the period.)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>For any bucket found public, list its objects and access logs for the exposure window. (Expect: The data exposed and any external access are identified.)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>All S3 buckets in the account (ListBuckets)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Agree the bucket count to the S3 console inventory for the account.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Full population</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>[DEMO DATA] 2026-01-01 to 2026-12-31 (assumed)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -589,7 +915,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>67d3b1ae-7dd2-49fb-b15f-3fce45051998</t>
+          <t>c057c748-a29c-4821-8cfd-33d034d284d7</t>
         </is>
       </c>
     </row>
@@ -625,7 +951,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-26T01:00:45+00:00</t>
+          <t>2026-09-26T22:31:08+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate screenshots, demo GIF and sample run after the demo fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEsj6q59UZDr5R4xFobVsY
</commit_message>
<xml_diff>
--- a/docs/sample-run/racm.xlsx
+++ b/docs/sample-run/racm.xlsx
@@ -768,7 +768,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[DEMO DATA] Customer data in S3 is exposed publicly.</t>
+          <t>[DEMO DATA] Data in S3 is exposed publicly.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A single public ACL exposes a bucket to the internet, and the buckets hold customer data.</t>
+          <t>A single public ACL exposes a bucket to the internet; the impact depends on the data held, which the data owner must confirm.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>c85898be-ad5a-4e0e-86f2-d2af3b62524b</t>
+          <t>713374ef-8db5-44be-9b4f-5470f1528ab0</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-26T22:51:25+00:00</t>
+          <t>2026-09-27T00:39:38+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the sample run and stop scanning its generated OSCAL for secrets
The sample report now carries the trail-verification line and the
conclusions-of-record block, and quotes still verify under session
binding. docs/sample-run/oscal.json is regenerated demo output whose
random vault ids tripped detect-secrets on every regeneration, so it is
excluded from that hook and its baseline entries are dropped.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEsj6q59UZDr5R4xFobVsY
</commit_message>
<xml_diff>
--- a/docs/sample-run/racm.xlsx
+++ b/docs/sample-run/racm.xlsx
@@ -915,7 +915,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4231ece5-08b7-41d7-bcce-acf273d10ac9</t>
+          <t>1a08dd3c-3c3d-4776-8599-a377a68523b5</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-27T21:00:30+00:00</t>
+          <t>2026-09-27T21:10:13+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>